<commit_message>
Add walk-forward backtest, drift filter, and revenue gate to earnings module
Earnings signals were the only module without historical validation — the bt dict
was faked with zeros. Now each candidate runs a 5-year walk-forward backtest using
yfinance earnings dates + price data (70/30 IS/OOS split, 6 quality gates).

New signal gates: revenue surprise consistency (gate 6), 10-day pre-earnings drift
filter to catch sell-the-news traps (gate 8), and short interest squeeze flag.
Backtest gates reject tickers where the strategy historically lost money (e.g. JPM).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_trades.xlsx
+++ b/paper_trades.xlsx
@@ -58,7 +58,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +69,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -94,6 +100,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +484,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-04-08 21:11</t>
+          <t>Last updated: 2026-04-10 12:31</t>
         </is>
       </c>
     </row>
@@ -635,7 +643,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -655,7 +663,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>0</v>
+        <v>7.66</v>
       </c>
     </row>
     <row r="26">
@@ -729,7 +737,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>0</v>
+        <v>7.66</v>
       </c>
     </row>
     <row r="36">
@@ -749,7 +757,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>0</v>
+        <v>7.66</v>
       </c>
     </row>
   </sheetData>
@@ -1120,7 +1128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1234,6 +1242,130 @@
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>20260408_earn_JPM</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>307.97</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>3.2471</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L2" s="7" t="n">
+        <v>310.33</v>
+      </c>
+      <c r="M2" s="8" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="N2" s="7" t="inlineStr"/>
+      <c r="O2" s="7" t="inlineStr"/>
+      <c r="P2" s="7" t="inlineStr"/>
+      <c r="Q2" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="R2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>20260410_earn_PEP</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>157.49</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>6.3496</v>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="n">
+        <v>157.49</v>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr"/>
+      <c r="P3" s="7" t="inlineStr"/>
+      <c r="Q3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix earnings entry timing, momentum vol filter, and Excel-CSV sync
- Add EARN_MIN_DAYS_BEFORE=2 to block same-day/next-day earnings entries
  that were gambling on announcements instead of riding anticipation
- Enforce minimum buffer in both live signal gate and backtest for consistency
- Widen earnings scan window to 5 days, backtest now matches live constraints
- Lower MOM_VOLUME_RATIO_MIN from 1.2 to 0.9 to filter collapsing volume
  without requiring a spike (was killing 94% of momentum candidates)
- Add CSV-to-Excel sync for all modules — Excel now picks up trade closures
  and missing entries from the authoritative CSV files on each daily run

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_trades.xlsx
+++ b/paper_trades.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +57,17 @@
       <color rgb="00006100"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +86,12 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -90,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -102,6 +117,12 @@
     <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,7 +505,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-04-10 12:31</t>
+          <t>Last updated: 2026-05-08 14:36</t>
         </is>
       </c>
     </row>
@@ -643,7 +664,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
@@ -663,7 +684,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>7.66</v>
+        <v>13.07</v>
       </c>
     </row>
     <row r="26">
@@ -737,7 +758,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>7.66</v>
+        <v>13.07</v>
       </c>
     </row>
     <row r="36">
@@ -757,7 +778,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>7.66</v>
+        <v>13.07</v>
       </c>
     </row>
   </sheetData>
@@ -1128,7 +1149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1244,128 +1265,714 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>20260408_earn_JPM</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>2026-04-08</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>JPM</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="12" t="n">
         <v>307.97</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="12" t="n">
         <v>3.2471</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="G2" s="12" t="n">
         <v>1000</v>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="I2" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>flat</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="n">
+        <v>316.99</v>
+      </c>
+      <c r="M2" s="13" t="inlineStr"/>
+      <c r="N2" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="O2" s="12" t="n">
+        <v>316.99</v>
+      </c>
+      <c r="P2" s="13" t="n">
+        <v>27.26</v>
+      </c>
+      <c r="Q2" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="R2" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>20260410_earn_PEP</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>157.49</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>6.3496</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>156.99</v>
+      </c>
+      <c r="M3" s="14" t="inlineStr"/>
+      <c r="N3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="n">
+        <v>156.99</v>
+      </c>
+      <c r="P3" s="14" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="Q3" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="R3" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>20260421_earn_BA</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>225.08</v>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>4.4429</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>231.28</v>
+      </c>
+      <c r="M4" s="13" t="inlineStr"/>
+      <c r="N4" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="O4" s="12" t="n">
+        <v>231.28</v>
+      </c>
+      <c r="P4" s="13" t="n">
+        <v>25.52</v>
+      </c>
+      <c r="Q4" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="R4" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>20260421_earn_GE</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>303.6</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>3.2938</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>281.47</v>
+      </c>
+      <c r="M5" s="13" t="inlineStr"/>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="O5" s="12" t="n">
+        <v>281.47</v>
+      </c>
+      <c r="P5" s="14" t="n">
+        <v>-74.81999999999999</v>
+      </c>
+      <c r="Q5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>20260422_earn_F</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>12.8413</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>77.8737</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>11.875</v>
+      </c>
+      <c r="M6" s="14" t="inlineStr"/>
+      <c r="N6" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>11.875</v>
+      </c>
+      <c r="P6" s="14" t="n">
+        <v>-77.17</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>20260422_earn_GM</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>79.45</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>12.5865</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>78.95</v>
+      </c>
+      <c r="M7" s="14" t="inlineStr"/>
+      <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="O7" s="12" t="n">
+        <v>78.95</v>
+      </c>
+      <c r="P7" s="14" t="n">
+        <v>-8.289999999999999</v>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>20260429_earn_AMZN</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>259.7</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>3.8506</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>growing</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>258.3808</v>
+      </c>
+      <c r="M8" s="13" t="inlineStr"/>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="O8" s="12" t="n">
+        <v>258.3808</v>
+      </c>
+      <c r="P8" s="14" t="n">
+        <v>-7.07</v>
+      </c>
+      <c r="Q8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>20260506_earn_CSCO</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>94.3</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>10.6045</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="L2" s="7" t="n">
-        <v>310.33</v>
-      </c>
-      <c r="M2" s="8" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="N2" s="7" t="inlineStr"/>
-      <c r="O2" s="7" t="inlineStr"/>
-      <c r="P2" s="7" t="inlineStr"/>
-      <c r="Q2" s="7" t="n">
+      <c r="L9" s="7" t="n">
+        <v>94.18000000000001</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr"/>
+      <c r="P9" s="7" t="inlineStr"/>
+      <c r="Q9" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="R2" s="7" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>20260410_earn_PEP</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>PEP</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="R9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>20260408_earn_WFC</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>WFC</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n">
-        <v>157.49</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>6.3496</v>
-      </c>
-      <c r="G3" s="7" t="n">
+      <c r="E10" s="12" t="n">
+        <v>84.66</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>11.812</v>
+      </c>
+      <c r="G10" s="12" t="n">
         <v>1000</v>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="n">
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="n">
         <v>75</v>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>growing</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>157.49</v>
-      </c>
-      <c r="M3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="7" t="inlineStr"/>
-      <c r="O3" s="7" t="inlineStr"/>
-      <c r="P3" s="7" t="inlineStr"/>
-      <c r="Q3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="7" t="inlineStr"/>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>81.97</v>
+      </c>
+      <c r="M10" s="12" t="inlineStr"/>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>81.97</v>
+      </c>
+      <c r="P10" s="14" t="n">
+        <v>-33.74</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>20260408_earn_GS</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>905.75</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>1.1041</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>flat</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>941.74</v>
+      </c>
+      <c r="M11" s="12" t="inlineStr"/>
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="n">
+        <v>941.74</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="Q11" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="R11" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix hold-day calc, harden FMP API, improve Excel sync, and add CLAUDE.md
Switch momentum and earnings hold_days from calendar days to business days
(np.busday_count) to match backtest bar counting. Add HTTP status handling
for FMP earnings API (402/non-200). Fix Excel momentum CSV sync to handle
open trades, not just closed. Use vol-targeting for momentum Excel entries.
Move API keys to env-var fallback. Rename header to ADF Trading System.
Clean up rotated logs.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_trades.xlsx
+++ b/paper_trades.xlsx
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 2026-05-08 14:36</t>
+          <t>Last updated: 2026-06-29 22:20</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0</v>
+        <v>20.36</v>
       </c>
     </row>
     <row r="16">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>13.07</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -693,8 +693,8 @@
           <t>Realized P/L:</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
+      <c r="B26" s="10" t="n">
+        <v>-37.58</v>
       </c>
     </row>
     <row r="28">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>13.07</v>
+        <v>56</v>
       </c>
     </row>
     <row r="36">
@@ -767,8 +767,8 @@
           <t>Total Realized:</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
-        <v>0</v>
+      <c r="B36" s="10" t="n">
+        <v>-17.22</v>
       </c>
     </row>
     <row r="37">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B37" s="6" t="n">
-        <v>13.07</v>
+        <v>38.78</v>
       </c>
     </row>
   </sheetData>
@@ -933,7 +933,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1029,6 +1029,361 @@
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>20260612_AMAT</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>552.64</v>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>1.8095</v>
+      </c>
+      <c r="G2" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="n">
+        <v>697.86</v>
+      </c>
+      <c r="J2" s="13" t="inlineStr"/>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="n">
+        <v>697.86</v>
+      </c>
+      <c r="M2" s="13" t="n">
+        <v>64.84999999999999</v>
+      </c>
+      <c r="N2" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="O2" s="12" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>20260612_STLD</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>279.55</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>3.5772</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>243.69</v>
+      </c>
+      <c r="J3" s="14" t="inlineStr"/>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>243.69</v>
+      </c>
+      <c r="M3" s="14" t="n">
+        <v>-44.49</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="O3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>20260613_INTC</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>124.57</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>8.0276</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>130.81</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>50.09</v>
+      </c>
+      <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr"/>
+      <c r="N4" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="O4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>20260620_CSCO</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>119.54</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>2.6022</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>311.07</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>117.71</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>-4.76</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="O5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>20260623_JBHT</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>JBHT</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>273.48</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>1.3362</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>365.43</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>284.685</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="inlineStr"/>
+      <c r="M6" s="7" t="inlineStr"/>
+      <c r="N6" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="O6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>20260625_STX</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>993.25</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>0.2517</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n">
+        <v>976.15</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>20260629_MU</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>1132.33</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0.2208</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>1132.33</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
+      <c r="M8" s="7" t="inlineStr"/>
+      <c r="N8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1769,66 +2124,76 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>20260506_earn_CSCO</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>CSCO</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>LONG</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="12" t="n">
         <v>94.3</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="12" t="n">
         <v>10.6045</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="12" t="n">
         <v>1000</v>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>2026-05-13</t>
         </is>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>flat</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>94.18000000000001</v>
-      </c>
-      <c r="M9" s="9" t="n">
-        <v>-1.27</v>
-      </c>
-      <c r="N9" s="7" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr"/>
-      <c r="P9" s="7" t="inlineStr"/>
-      <c r="Q9" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="R9" s="7" t="inlineStr"/>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>101.87</v>
+      </c>
+      <c r="M9" s="13" t="inlineStr"/>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="O9" s="12" t="n">
+        <v>101.87</v>
+      </c>
+      <c r="P9" s="13" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="Q9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
+        <is>
+          <t>post_earnings</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">

</xml_diff>